<commit_message>
Fix the AWS Continuum code review findings
- Stricter checks on saved answers: thread ids against the real list, dates
  in the normal format between 2020 and 2100, take-back items and flags that
  exist in the scenario, and unmeasurable bodies treated as too big. The
  follow-up date can no longer throw.
- Sign-up limits count +tag and Gmail-dot variations of an address as one,
  and a whole IPv6 /64 as one visitor (IPv4 unchanged).
- Short security notes (internal IDs only, never emails, links or internet
  addresses) for refused links, rate limits, refused requests, reader actions
  and button presses. Lambda logs kept 90 days.
- Privacy notice, privacy briefing and security review updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013sc1NQj5NJsvj6XwZ9CiCJ
</commit_message>
<xml_diff>
--- a/docs/app-text.xlsx
+++ b/docs/app-text.xlsx
@@ -18707,7 +18707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -18906,7 +18906,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Last updated: 26 October 2026.</t>
+          <t>Last updated: 27 October 2026.</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr"/>
@@ -18918,7 +18918,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;Last updated: 26 October 2026.&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;Last updated: 27 October 2026.&lt;"}</t>
         </is>
       </c>
     </row>
@@ -19381,12 +19381,12 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>paragraph</t>
+          <t>list item</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>We don't use cookies, tracking pixels, advertising or outside analytics, and we don't track whether you open our emails. While you have a file open, your browser keeps your personal link for that visit only, so the page can save your answers.</t>
+          <t>&lt;b&gt;Short security notes&lt;/b&gt;, so we can spot and look into misuse: for example, when a link is refused, when someone is blocked for trying too often, and when you confirm, pause, resume, unsubscribe or delete your data. They use our internal number for you, never your email address, your link or your internet address.</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr"/>
@@ -19398,7 +19398,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;We don't use cookies, tracking pixels, advertising or outside analytics, and we don't track whether you open our emails. While you have a file open, your browser keeps your personal link for that visit only, so the page can save your answers.&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;&lt;b&gt;Short security notes&lt;/b&gt;, so we can spot and look into misuse: for example, when a link is refused, when someone is blocked for trying too often, and when you confirm, pause, resume, unsubscribe or delete your data. They use our internal number for you, never your email address, your link or your internet address.&lt;"}</t>
         </is>
       </c>
     </row>
@@ -19413,12 +19413,12 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>heading</t>
+          <t>paragraph</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Our legal basis</t>
+          <t>We don't use cookies, tracking pixels, advertising or outside analytics, and we don't track whether you open our emails. While you have a file open, your browser keeps your personal link for that visit only, so the page can save your answers.</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr"/>
@@ -19430,7 +19430,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;Our legal basis&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;We don't use cookies, tracking pixels, advertising or outside analytics, and we don't track whether you open our emails. While you have a file open, your browser keeps your personal link for that visit only, so the page can save your answers.&lt;"}</t>
         </is>
       </c>
     </row>
@@ -19445,12 +19445,12 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>paragraph</t>
+          <t>heading</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>We rely on your consent, which you give when you sign up and confirm your email. It covers the monthly emails, keeping your answers and flight recorder, and recording which screens you reach so we can improve the scenarios.</t>
+          <t>Our legal basis</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr"/>
@@ -19462,7 +19462,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;We rely on your consent, which you give when you sign up and confirm your email. It covers the monthly emails, keeping your answers and flight recorder, and recording which screens you reach so we can improve the scenarios.&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;Our legal basis&lt;"}</t>
         </is>
       </c>
     </row>
@@ -19482,7 +19482,7 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>You can withdraw your consent at any time using the link at the bottom of any of our emails. To stop the emails, unsubscribe. To withdraw your consent completely, delete your data, and we'll remove everything straight away.</t>
+          <t>We rely on your consent, which you give when you sign up and confirm your email. It covers the monthly emails, keeping your answers and flight recorder, and recording which screens you reach so we can improve the scenarios.</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr"/>
@@ -19494,7 +19494,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;You can withdraw your consent at any time using the link at the bottom of any of our emails. To stop the emails, unsubscribe. To withdraw your consent completely, delete your data, and we'll remove everything straight away.&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;We rely on your consent, which you give when you sign up and confirm your email. It covers the monthly emails, keeping your answers and flight recorder, and recording which screens you reach so we can improve the scenarios.&lt;"}</t>
         </is>
       </c>
     </row>
@@ -19509,12 +19509,12 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>heading</t>
+          <t>paragraph</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Who else handles your data</t>
+          <t>You can withdraw your consent at any time using the link at the bottom of any of our emails. To stop the emails, unsubscribe. To withdraw your consent completely, delete your data, and we'll remove everything straight away.</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr"/>
@@ -19526,7 +19526,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;Who else handles your data&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;You can withdraw your consent at any time using the link at the bottom of any of our emails. To stop the emails, unsubscribe. To withdraw your consent completely, delete your data, and we'll remove everything straight away.&lt;"}</t>
         </is>
       </c>
     </row>
@@ -19541,12 +19541,12 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>list item</t>
+          <t>heading</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>&lt;b&gt;Amazon Web Services (AWS)&lt;/b&gt; runs the website, stores the data and sends our emails, acting only on our instructions. Your data is stored in AWS's London region. To make pages load quickly, AWS may handle your visit at its nearest location in Europe or North America.</t>
+          <t>Who else handles your data</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr"/>
@@ -19558,7 +19558,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;&lt;b&gt;Amazon Web Services (AWS)&lt;/b&gt; runs the website, stores the data and sends our emails, acting only on our instructions. Your data is stored in AWS's London region. To make pages load quickly, AWS may handle your visit at its nearest location in Europe or North America.&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;Who else handles your data&lt;"}</t>
         </is>
       </c>
     </row>
@@ -19578,7 +19578,7 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>&lt;b&gt;Google Workspace&lt;/b&gt; holds our email inbox. If you reply to one of our emails, your reply is kept there.</t>
+          <t>&lt;b&gt;Amazon Web Services (AWS)&lt;/b&gt; runs the website, stores the data and sends our emails, acting only on our instructions. Your data is stored in AWS's London region. To make pages load quickly, AWS may handle your visit at its nearest location in Europe or North America.</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr"/>
@@ -19590,7 +19590,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;&lt;b&gt;Google Workspace&lt;/b&gt; holds our email inbox. If you reply to one of our emails, your reply is kept there.&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;&lt;b&gt;Amazon Web Services (AWS)&lt;/b&gt; runs the website, stores the data and sends our emails, acting only on our instructions. Your data is stored in AWS's London region. To make pages load quickly, AWS may handle your visit at its nearest location in Europe or North America.&lt;"}</t>
         </is>
       </c>
     </row>
@@ -19605,12 +19605,12 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>paragraph</t>
+          <t>list item</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>We never sell your data or share it with anyone else, unless the law requires it.</t>
+          <t>&lt;b&gt;Google Workspace&lt;/b&gt; holds our email inbox. If you reply to one of our emails, your reply is kept there.</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr"/>
@@ -19622,7 +19622,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;We never sell your data or share it with anyone else, unless the law requires it.&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;&lt;b&gt;Google Workspace&lt;/b&gt; holds our email inbox. If you reply to one of our emails, your reply is kept there.&lt;"}</t>
         </is>
       </c>
     </row>
@@ -19637,12 +19637,12 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>heading</t>
+          <t>paragraph</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>How long we keep it</t>
+          <t>We never sell your data or share it with anyone else, unless the law requires it.</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr"/>
@@ -19654,7 +19654,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;How long we keep it&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;We never sell your data or share it with anyone else, unless the law requires it.&lt;"}</t>
         </is>
       </c>
     </row>
@@ -19669,12 +19669,12 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>list item</t>
+          <t>heading</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>&lt;b&gt;If you don't confirm your email:&lt;/b&gt; we delete your sign-up after 7 days.</t>
+          <t>How long we keep it</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr"/>
@@ -19686,7 +19686,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;&lt;b&gt;If you don't confirm your email:&lt;/b&gt; we delete your sign-up after 7 days.&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;How long we keep it&lt;"}</t>
         </is>
       </c>
     </row>
@@ -19706,7 +19706,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>&lt;b&gt;Everything else:&lt;/b&gt; we delete it 2 years after you last opened one of our files. Unsubscribing stops the emails; your past answers are then deleted 2 years after you last took part.</t>
+          <t>&lt;b&gt;If you don't confirm your email:&lt;/b&gt; we delete your sign-up after 7 days.</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr"/>
@@ -19718,7 +19718,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;&lt;b&gt;Everything else:&lt;/b&gt; we delete it 2 years after you last opened one of our files. Unsubscribing stops the emails; your past answers are then deleted 2 years after you last took part.&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;&lt;b&gt;If you don't confirm your email:&lt;/b&gt; we delete your sign-up after 7 days.&lt;"}</t>
         </is>
       </c>
     </row>
@@ -19738,7 +19738,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>&lt;b&gt;If you ask us to delete your data:&lt;/b&gt; it's removed from the service straight away. Our backups, which let us recover from mistakes, keep a copy for up to 35 days before it disappears for good.</t>
+          <t>&lt;b&gt;Everything else:&lt;/b&gt; we delete it 2 years after you last opened one of our files. Unsubscribing stops the emails; your past answers are then deleted 2 years after you last took part.</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr"/>
@@ -19750,7 +19750,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;&lt;b&gt;If you ask us to delete your data:&lt;/b&gt; it's removed from the service straight away. Our backups, which let us recover from mistakes, keep a copy for up to 35 days before it disappears for good.&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;&lt;b&gt;Everything else:&lt;/b&gt; we delete it 2 years after you last opened one of our files. Unsubscribing stops the emails; your past answers are then deleted 2 years after you last took part.&lt;"}</t>
         </is>
       </c>
     </row>
@@ -19770,7 +19770,7 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>&lt;b&gt;Replies you send us&lt;/b&gt; stay in our inbox until we delete them.</t>
+          <t>&lt;b&gt;If you ask us to delete your data:&lt;/b&gt; it's removed from the service straight away. Our backups, which let us recover from mistakes, keep a copy for up to 35 days before it disappears for good.</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr"/>
@@ -19782,7 +19782,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;&lt;b&gt;Replies you send us&lt;/b&gt; stay in our inbox until we delete them.&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;&lt;b&gt;If you ask us to delete your data:&lt;/b&gt; it's removed from the service straight away. Our backups, which let us recover from mistakes, keep a copy for up to 35 days before it disappears for good.&lt;"}</t>
         </is>
       </c>
     </row>
@@ -19802,7 +19802,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>&lt;b&gt;If an email to you bounces or is marked as spam,&lt;/b&gt; AWS keeps your address on a "do not send" list so we don't email you again.</t>
+          <t>&lt;b&gt;Security notes&lt;/b&gt; are deleted after 90 days. This includes the note that you deleted your data, which shows it was done.</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr"/>
@@ -19814,7 +19814,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;&lt;b&gt;If an email to you bounces or is marked as spam,&lt;/b&gt; AWS keeps your address on a \"do not send\" list so we don't email you again.&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;&lt;b&gt;Security notes&lt;/b&gt; are deleted after 90 days. This includes the note that you deleted your data, which shows it was done.&lt;"}</t>
         </is>
       </c>
     </row>
@@ -19829,12 +19829,12 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>heading</t>
+          <t>list item</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Your rights</t>
+          <t>&lt;b&gt;Replies you send us&lt;/b&gt; stay in our inbox until we delete them.</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr"/>
@@ -19846,7 +19846,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;Your rights&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;&lt;b&gt;Replies you send us&lt;/b&gt; stay in our inbox until we delete them.&lt;"}</t>
         </is>
       </c>
     </row>
@@ -19861,12 +19861,12 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>paragraph</t>
+          <t>list item</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>You can ask to see the data we hold about you, have it corrected or deleted, limit how we use it, object to how we use it, or receive a copy to take elsewhere. You can take a 3-month break, unsubscribe, or delete everything at once using the link at the bottom of any of our emails. For anything else, reply to any email or write to the address above. We'll respond within a month.</t>
+          <t>&lt;b&gt;If an email to you bounces or is marked as spam,&lt;/b&gt; AWS keeps your address on a "do not send" list so we don't email you again.</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr"/>
@@ -19878,7 +19878,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;You can ask to see the data we hold about you, have it corrected or deleted, limit how we use it, object to how we use it, or receive a copy to take elsewhere. You can take a 3-month break, unsubscribe, or delete everything at once using the link at the bottom of any of our emails. For anything else, reply to any email or write to the address above. We'll respond within a month.&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;&lt;b&gt;If an email to you bounces or is marked as spam,&lt;/b&gt; AWS keeps your address on a \"do not send\" list so we don't email you again.&lt;"}</t>
         </is>
       </c>
     </row>
@@ -19893,12 +19893,12 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>paragraph</t>
+          <t>heading</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>If you're unhappy with how we've handled your data, please tell us first. You can also complain to the Information Commissioner's Office (ICO) at &lt;a href="https://ico.org.uk/make-a-complaint/"&gt;ico.org.uk/make-a-complaint&lt;/a&gt;.</t>
+          <t>Your rights</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr"/>
@@ -19910,7 +19910,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;If you're unhappy with how we've handled your data, please tell us first. You can also complain to the Information Commissioner's Office (ICO) at &lt;a href=\"https://ico.org.uk/make-a-complaint/\"&gt;ico.org.uk/make-a-complaint&lt;/a&gt;.&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;Your rights&lt;"}</t>
         </is>
       </c>
     </row>
@@ -19925,12 +19925,12 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>heading</t>
+          <t>paragraph</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Changes</t>
+          <t>You can ask to see the data we hold about you, have it corrected or deleted, limit how we use it, object to how we use it, or receive a copy to take elsewhere. You can take a 3-month break, unsubscribe, or delete everything at once using the link at the bottom of any of our emails. For anything else, reply to any email or write to the address above. We'll respond within a month.</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr"/>
@@ -19942,7 +19942,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;Changes&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;You can ask to see the data we hold about you, have it corrected or deleted, limit how we use it, object to how we use it, or receive a copy to take elsewhere. You can take a 3-month break, unsubscribe, or delete everything at once using the link at the bottom of any of our emails. For anything else, reply to any email or write to the address above. We'll respond within a month.&lt;"}</t>
         </is>
       </c>
     </row>
@@ -19962,7 +19962,7 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>If we change how we use your data, we'll update this page and change the date at the top. If a change is significant, we'll tell you by email first.</t>
+          <t>If you're unhappy with how we've handled your data, please tell us first. You can also complain to the Information Commissioner's Office (ICO) at &lt;a href="https://ico.org.uk/make-a-complaint/"&gt;ico.org.uk/make-a-complaint&lt;/a&gt;.</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr"/>
@@ -19974,7 +19974,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;If we change how we use your data, we'll update this page and change the date at the top. If a change is significant, we'll tell you by email first.&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;If you're unhappy with how we've handled your data, please tell us first. You can also complain to the Information Commissioner's Office (ICO) at &lt;a href=\"https://ico.org.uk/make-a-complaint/\"&gt;ico.org.uk/make-a-complaint&lt;/a&gt;.&lt;"}</t>
         </is>
       </c>
     </row>
@@ -19989,12 +19989,12 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>link</t>
+          <t>heading</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Back to The Monday After</t>
+          <t>Changes</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr"/>
@@ -20005,6 +20005,70 @@
         </is>
       </c>
       <c r="H40" t="inlineStr">
+        <is>
+          <t>{"kind": "text", "raw": "&gt;Changes&lt;"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Privacy notice</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>paragraph</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>If we change how we use your data, we'll update this page and change the date at the top. If a change is significant, we'll tell you by email first.</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr"/>
+      <c r="F41" s="3" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>site/privacy.html</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>{"kind": "text", "raw": "&gt;If we change how we use your data, we'll update this page and change the date at the top. If a change is significant, we'll tell you by email first.&lt;"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="n">
+        <v>601</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Privacy notice</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Back to The Monday After</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr"/>
+      <c r="F42" s="3" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>site/privacy.html</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
         <is>
           <t>{"kind": "text", "raw": "&gt;Back to The Monday After&lt;"}</t>
         </is>

</xml_diff>

<commit_message>
Owner's wording decisions: dependency and trust lines, punctuation tidy, sign-up teaser matches the email
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013sc1NQj5NJsvj6XwZ9CiCJ
</commit_message>
<xml_diff>
--- a/docs/app-text.xlsx
+++ b/docs/app-text.xlsx
@@ -786,7 +786,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>The contract sits with HR. IT has never seen it. Your organisation doesn't have a list of its contractors</t>
+          <t>The contract sits with HR. IT has never seen it. Your organisation doesn't have a list of its contractors.</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr"/>
@@ -1618,7 +1618,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Pick one or two. Your answers shape what happens next</t>
+          <t>Pick one or two. Your answers shape what happens next.</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr"/>
@@ -2642,7 +2642,7 @@
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>You can have a sensible conversation with workers representatives. Your proactive approach will be welcomed and they won't use the opportunity to increase tensions in the relationship.</t>
+          <t>You can have a sensible conversation with workers’ representatives. Your proactive approach will be welcomed and they won't use the opportunity to increase tensions in the relationship.</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr"/>
@@ -2898,7 +2898,7 @@
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Identify the mission critical work, and model the impact of reduced capacity on service levels.</t>
+          <t>Identify the mission-critical work, and model the impact of reduced capacity on service levels.</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr"/>
@@ -3218,7 +3218,7 @@
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>This is HR’s problem.</t>
+          <t>This is HR’s problem</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr"/>
@@ -4850,7 +4850,7 @@
       </c>
       <c r="D135" s="3" t="inlineStr">
         <is>
-          <t>Because you built the list, you can deal directly with contractors and make short term arrangements.</t>
+          <t>Because you built the list, you can deal directly with contractors and make short-term arrangements.</t>
         </is>
       </c>
       <c r="E135" s="4" t="inlineStr"/>
@@ -4978,7 +4978,7 @@
       </c>
       <c r="D139" s="3" t="inlineStr">
         <is>
-          <t>Brief the workers</t>
+          <t>Brief the workers.</t>
         </is>
       </c>
       <c r="E139" s="4" t="inlineStr"/>
@@ -5010,7 +5010,7 @@
       </c>
       <c r="D140" s="3" t="inlineStr">
         <is>
-          <t>Tell the workers what you do and don't know.</t>
+          <t>Tell the workers what you do and don't know</t>
         </is>
       </c>
       <c r="E140" s="4" t="inlineStr"/>
@@ -5074,7 +5074,7 @@
       </c>
       <c r="D142" s="3" t="inlineStr">
         <is>
-          <t>Escalate</t>
+          <t>Escalate.</t>
         </is>
       </c>
       <c r="E142" s="4" t="inlineStr"/>
@@ -6642,7 +6642,7 @@
       </c>
       <c r="D191" s="3" t="inlineStr">
         <is>
-          <t>Nobody has mapped what else those contractors can reach, and the same agency still supplies them.</t>
+          <t>Nobody has mapped the organisation’s dependence on contractors.</t>
         </is>
       </c>
       <c r="E191" s="4" t="inlineStr"/>
@@ -6674,7 +6674,7 @@
       </c>
       <c r="D192" s="3" t="inlineStr">
         <is>
-          <t>The next failure exposes similar supply chain dependencies, gaps in your data and dependence on contractors</t>
+          <t>The next failure exposes similar supply chain dependencies, gaps in your data and dependence on contractors.</t>
         </is>
       </c>
       <c r="E192" s="4" t="inlineStr"/>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="D197" s="3" t="inlineStr">
         <is>
-          <t>Your only route to these workers was one agency. It was dependent on one provider. One failed so they both failed.</t>
+          <t>Your only route to these workers was one agency. It was dependent on one provider. One failed, so they both failed.</t>
         </is>
       </c>
       <c r="E197" s="4" t="inlineStr"/>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="D210" s="3" t="inlineStr">
         <is>
-          <t>The HR team is better-placed to manage its suppliers</t>
+          <t>The HR team is better placed to manage its suppliers.</t>
         </is>
       </c>
       <c r="E210" s="4" t="inlineStr"/>
@@ -7602,7 +7602,7 @@
       </c>
       <c r="D221" s="3" t="inlineStr">
         <is>
-          <t>IT is firmly in charge but can it reduce risk?</t>
+          <t>IT is firmly in charge, but can it reduce risk?</t>
         </is>
       </c>
       <c r="E221" s="4" t="inlineStr"/>
@@ -7666,7 +7666,7 @@
       </c>
       <c r="D223" s="3" t="inlineStr">
         <is>
-          <t>Finance HR and IT have collaborated successfully and can again</t>
+          <t>Finance, HR and IT worked together successfully and value IT’s governance processes more highly. How can you use that to increase compliance across the organisation?</t>
         </is>
       </c>
       <c r="E223" s="4" t="inlineStr"/>
@@ -15926,7 +15926,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Your temps and contractors haven't been paid. Nobody will say why.</t>
+          <t>Your temps and contractors haven't been paid. Nobody knows why.</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr"/>
@@ -15938,7 +15938,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;Your temps and contractors haven't been paid. Nobody will say why.&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;Your temps and contractors haven't been paid. Nobody knows why.&lt;"}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Say 'The Monday After team' instead of 'the author' in the privacy lines
Flight recorder screen, forecast screen and the flight recorder email.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013sc1NQj5NJsvj6XwZ9CiCJ
</commit_message>
<xml_diff>
--- a/docs/app-text.xlsx
+++ b/docs/app-text.xlsx
@@ -5618,7 +5618,7 @@
       </c>
       <c r="D159" s="3" t="inlineStr">
         <is>
-          <t>No names or confidential detail. Write it as a pattern. Private to you: encrypted, and the author can’t read it. Timestamped, saved before the ledger.</t>
+          <t>No names or confidential detail. Write it as a pattern. Encrypted and private to you: The Monday After team can’t read it. Timestamped, saved before the ledger.</t>
         </is>
       </c>
       <c r="E159" s="4" t="inlineStr"/>
@@ -6194,7 +6194,7 @@
       </c>
       <c r="D177" s="3" t="inlineStr">
         <is>
-          <t>Only you and the author see your forecast.</t>
+          <t>Only you and The Monday After team see your forecast.</t>
         </is>
       </c>
       <c r="E177" s="4" t="inlineStr"/>
@@ -18744,7 +18744,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Only you can see this. The author of </t>
+          <t xml:space="preserve">Only you can see this. </t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr"/>
@@ -18756,7 +18756,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\"Only you can see this. The author of \""}</t>
+          <t>{"kind": "code", "raw": "\"Only you can see this. \""}</t>
         </is>
       </c>
     </row>
@@ -18776,7 +18776,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> can't read your flight recorder.</t>
+          <t xml:space="preserve"> team can't read your flight recorder.</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr"/>
@@ -18788,7 +18788,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\" can't read your flight recorder.\""}</t>
+          <t>{"kind": "code", "raw": "\" team can't read your flight recorder.\""}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build the 30-day follow-up, the check before every send, and Option A
- 30-day follow-up: a daily job emails readers who asked, once each, with a
  link to a Yes / Partly / Not yet page (followup.html). Answers are kept on
  the reader's answers record and appear in the exports.
- Before Send Incident File and the follow-ups, SES account status and the
  bounce and complaint rates are checked; nothing is sent at 4% bounces or
  0.08% complaints. The Send summary shows the rates.
- Option A: the current copy keeps its tables, key and logs if the code is
  ever removed, with deletion protection on the tables.
- The bare web address shows the sign-up page; Share shares the sign-up page.
- Pen test finished: remove the AWS Security Agent verification file.
- Privacy notice and wording spreadsheet updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013sc1NQj5NJsvj6XwZ9CiCJ
</commit_message>
<xml_diff>
--- a/docs/app-text.xlsx
+++ b/docs/app-text.xlsx
@@ -14669,7 +14669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -16042,7 +16042,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Message · expired link</t>
+          <t>Follow-up page · expired link</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -16052,19 +16052,19 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>This link has expired or isn't valid. Reply to any Monday After email and we'll send you a fresh one.</t>
+          <t>This link has expired or isn't valid. Reply to any Monday After email if you'd like to tell us anyway.</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr"/>
       <c r="F43" s="3" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>backend/src/service.ts</t>
+          <t>site/js/pages.js</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\"This link has expired or isn't valid. Reply to any Monday After email and we'll send you a fresh one.\""}</t>
+          <t>{"kind": "code", "raw": "\"This link has expired or isn't valid. Reply to any Monday After email if you'd like to tell us anyway.\""}</t>
         </is>
       </c>
     </row>
@@ -16074,7 +16074,7 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Message · too many tries</t>
+          <t>Follow-up page · after answering Yes</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
@@ -16084,19 +16084,19 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Too many requests. Please wait a little and try again.</t>
+          <t>You did it.</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr"/>
       <c r="F44" s="3" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>backend/src/service.ts</t>
+          <t>site/js/pages.js</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\"Too many requests. Please wait a little and try again.\""}</t>
+          <t>{"kind": "code", "raw": "\"You did it.\""}</t>
         </is>
       </c>
     </row>
@@ -16106,7 +16106,7 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Sign-up page · busy</t>
+          <t>Follow-up page · after answering Partly</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
@@ -16116,19 +16116,19 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>We're getting a lot of sign-ups right now. Please try again in an hour.</t>
+          <t>You did part of it.</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr"/>
       <c r="F45" s="3" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>backend/src/service.ts</t>
+          <t>site/js/pages.js</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\"We're getting a lot of sign-ups right now. Please try again in an hour.\""}</t>
+          <t>{"kind": "code", "raw": "\"You did part of it.\""}</t>
         </is>
       </c>
     </row>
@@ -16138,7 +16138,7 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>App · email me my flight recorder, nothing saved</t>
+          <t>Follow-up page · after answering Not yet</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -16148,19 +16148,19 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>There's no saved flight recorder for this file.</t>
+          <t>Not yet.</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr"/>
       <c r="F46" s="3" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>backend/src/service.ts</t>
+          <t>site/js/pages.js</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\"There's no saved flight recorder for this file.\""}</t>
+          <t>{"kind": "code", "raw": "\"Not yet.\""}</t>
         </is>
       </c>
     </row>
@@ -16170,7 +16170,7 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Manage page</t>
+          <t>Follow-up page · after answering (end)</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -16180,19 +16180,19 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>You're unsubscribed, so there's nothing to pause.</t>
+          <t xml:space="preserve"> That's saved with your answers for this file.</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr"/>
       <c r="F47" s="3" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>backend/src/service.ts</t>
+          <t>site/js/pages.js</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\"You're unsubscribed, so there's nothing to pause.\""}</t>
+          <t>{"kind": "code", "raw": "\" That's saved with your answers for this file.\""}</t>
         </is>
       </c>
     </row>
@@ -16202,7 +16202,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Sign-up page · empty email</t>
+          <t>Follow-up page (then the file name)</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -16212,19 +16212,19 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Email is missing</t>
+          <t xml:space="preserve">30 days ago, at the end of </t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr"/>
       <c r="F48" s="3" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>backend/src/validate.ts</t>
+          <t>site/js/pages.js</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\"Email is missing\""}</t>
+          <t>{"kind": "code", "raw": "\"30 days ago, at the end of \""}</t>
         </is>
       </c>
     </row>
@@ -16234,7 +16234,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Sign-up page · bad email</t>
+          <t>Follow-up page (end)</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -16244,19 +16244,19 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>That doesn't look like an email address</t>
+          <t>, you chose one thing to take back.</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr"/>
       <c r="F49" s="3" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>backend/src/validate.ts</t>
+          <t>site/js/pages.js</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\"That doesn't look like an email address\""}</t>
+          <t>{"kind": "code", "raw": "\", you chose one thing to take back.\""}</t>
         </is>
       </c>
     </row>
@@ -16266,7 +16266,7 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Flight recorder · too long (then a number)</t>
+          <t>Follow-up page · answers deleted</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -16276,19 +16276,19 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Please keep each entry under </t>
+          <t>There's nothing to answer for this file any more.</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr"/>
       <c r="F50" s="3" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>backend/src/validate.ts</t>
+          <t>backend/src/service.ts</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\"Please keep each entry under \""}</t>
+          <t>{"kind": "code", "raw": "\"There's nothing to answer for this file any more.\""}</t>
         </is>
       </c>
     </row>
@@ -16298,7 +16298,7 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Flight recorder · first hour empty</t>
+          <t>Follow-up page</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -16308,17 +16308,305 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Please write something for the first hour</t>
+          <t>Please choose one of the answers.</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr"/>
       <c r="F51" s="3" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
+          <t>backend/src/service.ts</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>{"kind": "code", "raw": "\"Please choose one of the answers.\""}</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="n">
+        <v>491</v>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Message · expired link</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>This link has expired or isn't valid. Reply to any Monday After email and we'll send you a fresh one.</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr"/>
+      <c r="F52" s="3" t="inlineStr"/>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>backend/src/service.ts</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>{"kind": "code", "raw": "\"This link has expired or isn't valid. Reply to any Monday After email and we'll send you a fresh one.\""}</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="n">
+        <v>492</v>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Message · too many tries</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Too many requests. Please wait a little and try again.</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr"/>
+      <c r="F53" s="3" t="inlineStr"/>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>backend/src/service.ts</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>{"kind": "code", "raw": "\"Too many requests. Please wait a little and try again.\""}</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="n">
+        <v>493</v>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Sign-up page · busy</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>We're getting a lot of sign-ups right now. Please try again in an hour.</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr"/>
+      <c r="F54" s="3" t="inlineStr"/>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>backend/src/service.ts</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>{"kind": "code", "raw": "\"We're getting a lot of sign-ups right now. Please try again in an hour.\""}</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="n">
+        <v>494</v>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>App · email me my flight recorder, nothing saved</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>There's no saved flight recorder for this file.</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr"/>
+      <c r="F55" s="3" t="inlineStr"/>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>backend/src/service.ts</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>{"kind": "code", "raw": "\"There's no saved flight recorder for this file.\""}</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="n">
+        <v>495</v>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Manage page</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>You're unsubscribed, so there's nothing to pause.</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr"/>
+      <c r="F56" s="3" t="inlineStr"/>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>backend/src/service.ts</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>{"kind": "code", "raw": "\"You're unsubscribed, so there's nothing to pause.\""}</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="n">
+        <v>496</v>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Sign-up page · empty email</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Email is missing</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr"/>
+      <c r="F57" s="3" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
+        <is>
           <t>backend/src/validate.ts</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr">
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>{"kind": "code", "raw": "\"Email is missing\""}</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="n">
+        <v>497</v>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Sign-up page · bad email</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>That doesn't look like an email address</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr"/>
+      <c r="F58" s="3" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>backend/src/validate.ts</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>{"kind": "code", "raw": "\"That doesn't look like an email address\""}</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="n">
+        <v>498</v>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Flight recorder · too long (then a number)</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Please keep each entry under </t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr"/>
+      <c r="F59" s="3" t="inlineStr"/>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>backend/src/validate.ts</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>{"kind": "code", "raw": "\"Please keep each entry under \""}</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="n">
+        <v>499</v>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Flight recorder · first hour empty</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>Please write something for the first hour</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr"/>
+      <c r="F60" s="3" t="inlineStr"/>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>backend/src/validate.ts</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
         <is>
           <t>{"kind": "code", "raw": "\"Please write something for the first hour\""}</t>
         </is>
@@ -16335,7 +16623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H80"/>
+  <dimension ref="A1:H95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -16392,7 +16680,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
-        <v>491</v>
+        <v>500</v>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
@@ -16424,7 +16712,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
-        <v>492</v>
+        <v>501</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
@@ -16456,7 +16744,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
-        <v>493</v>
+        <v>502</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
@@ -16488,7 +16776,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
-        <v>494</v>
+        <v>503</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -16520,7 +16808,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
-        <v>495</v>
+        <v>504</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
@@ -16552,7 +16840,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
-        <v>496</v>
+        <v>505</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
@@ -16584,7 +16872,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
-        <v>497</v>
+        <v>506</v>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
@@ -16616,7 +16904,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
-        <v>498</v>
+        <v>507</v>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
@@ -16648,7 +16936,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
-        <v>499</v>
+        <v>508</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
@@ -16680,7 +16968,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
-        <v>500</v>
+        <v>509</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
@@ -16712,7 +17000,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
-        <v>501</v>
+        <v>510</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
@@ -16744,7 +17032,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
-        <v>502</v>
+        <v>511</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
@@ -16776,7 +17064,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
-        <v>503</v>
+        <v>512</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
@@ -16808,7 +17096,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
-        <v>504</v>
+        <v>513</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
@@ -16840,7 +17128,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
-        <v>505</v>
+        <v>514</v>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
@@ -16872,7 +17160,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
-        <v>506</v>
+        <v>515</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
@@ -16904,7 +17192,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
-        <v>507</v>
+        <v>516</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
@@ -16936,7 +17224,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
-        <v>508</v>
+        <v>517</v>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
@@ -16968,7 +17256,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
-        <v>509</v>
+        <v>518</v>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
@@ -17000,7 +17288,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
-        <v>510</v>
+        <v>519</v>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
@@ -17032,7 +17320,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
-        <v>511</v>
+        <v>520</v>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
@@ -17064,7 +17352,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
-        <v>512</v>
+        <v>521</v>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
@@ -17096,7 +17384,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
-        <v>513</v>
+        <v>522</v>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
@@ -17128,7 +17416,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
-        <v>514</v>
+        <v>523</v>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
@@ -17160,7 +17448,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
-        <v>515</v>
+        <v>524</v>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
@@ -17192,7 +17480,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
-        <v>516</v>
+        <v>525</v>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
@@ -17224,7 +17512,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
-        <v>517</v>
+        <v>526</v>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
@@ -17256,7 +17544,7 @@
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
-        <v>518</v>
+        <v>527</v>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
@@ -17288,7 +17576,7 @@
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
-        <v>519</v>
+        <v>528</v>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
@@ -17320,7 +17608,7 @@
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
-        <v>520</v>
+        <v>529</v>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
@@ -17352,7 +17640,7 @@
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
-        <v>521</v>
+        <v>530</v>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
@@ -17384,7 +17672,7 @@
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
-        <v>522</v>
+        <v>531</v>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
@@ -17416,7 +17704,7 @@
     </row>
     <row r="34">
       <c r="A34" s="3" t="n">
-        <v>523</v>
+        <v>532</v>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
@@ -17448,7 +17736,7 @@
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
-        <v>524</v>
+        <v>533</v>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
@@ -17480,7 +17768,7 @@
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
-        <v>525</v>
+        <v>534</v>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
@@ -17512,7 +17800,7 @@
     </row>
     <row r="37">
       <c r="A37" s="3" t="n">
-        <v>526</v>
+        <v>535</v>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
@@ -17544,7 +17832,7 @@
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
-        <v>527</v>
+        <v>536</v>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
@@ -17576,7 +17864,7 @@
     </row>
     <row r="39">
       <c r="A39" s="3" t="n">
-        <v>528</v>
+        <v>537</v>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
@@ -17608,7 +17896,7 @@
     </row>
     <row r="40">
       <c r="A40" s="3" t="n">
-        <v>529</v>
+        <v>538</v>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
@@ -17640,7 +17928,7 @@
     </row>
     <row r="41">
       <c r="A41" s="3" t="n">
-        <v>530</v>
+        <v>539</v>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
@@ -17672,7 +17960,7 @@
     </row>
     <row r="42">
       <c r="A42" s="3" t="n">
-        <v>531</v>
+        <v>540</v>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
@@ -17704,7 +17992,7 @@
     </row>
     <row r="43">
       <c r="A43" s="3" t="n">
-        <v>532</v>
+        <v>541</v>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
@@ -17736,7 +18024,7 @@
     </row>
     <row r="44">
       <c r="A44" s="3" t="n">
-        <v>533</v>
+        <v>542</v>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
@@ -17768,7 +18056,7 @@
     </row>
     <row r="45">
       <c r="A45" s="3" t="n">
-        <v>534</v>
+        <v>543</v>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
@@ -17800,7 +18088,7 @@
     </row>
     <row r="46">
       <c r="A46" s="3" t="n">
-        <v>535</v>
+        <v>544</v>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
@@ -17832,7 +18120,7 @@
     </row>
     <row r="47">
       <c r="A47" s="3" t="n">
-        <v>536</v>
+        <v>545</v>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
@@ -17864,7 +18152,7 @@
     </row>
     <row r="48">
       <c r="A48" s="3" t="n">
-        <v>537</v>
+        <v>546</v>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
@@ -17896,7 +18184,7 @@
     </row>
     <row r="49">
       <c r="A49" s="3" t="n">
-        <v>538</v>
+        <v>547</v>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
@@ -17928,7 +18216,7 @@
     </row>
     <row r="50">
       <c r="A50" s="3" t="n">
-        <v>539</v>
+        <v>548</v>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
@@ -17960,7 +18248,7 @@
     </row>
     <row r="51">
       <c r="A51" s="3" t="n">
-        <v>540</v>
+        <v>549</v>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
@@ -17992,7 +18280,7 @@
     </row>
     <row r="52">
       <c r="A52" s="3" t="n">
-        <v>541</v>
+        <v>550</v>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
@@ -18024,7 +18312,7 @@
     </row>
     <row r="53">
       <c r="A53" s="3" t="n">
-        <v>542</v>
+        <v>551</v>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
@@ -18056,7 +18344,7 @@
     </row>
     <row r="54">
       <c r="A54" s="3" t="n">
-        <v>543</v>
+        <v>552</v>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
@@ -18088,7 +18376,7 @@
     </row>
     <row r="55">
       <c r="A55" s="3" t="n">
-        <v>544</v>
+        <v>553</v>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
@@ -18120,7 +18408,7 @@
     </row>
     <row r="56">
       <c r="A56" s="3" t="n">
-        <v>545</v>
+        <v>554</v>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
@@ -18152,7 +18440,7 @@
     </row>
     <row r="57">
       <c r="A57" s="3" t="n">
-        <v>546</v>
+        <v>555</v>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
@@ -18184,7 +18472,7 @@
     </row>
     <row r="58">
       <c r="A58" s="3" t="n">
-        <v>547</v>
+        <v>556</v>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
@@ -18216,7 +18504,7 @@
     </row>
     <row r="59">
       <c r="A59" s="3" t="n">
-        <v>548</v>
+        <v>557</v>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
@@ -18248,7 +18536,7 @@
     </row>
     <row r="60">
       <c r="A60" s="3" t="n">
-        <v>549</v>
+        <v>558</v>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
@@ -18280,7 +18568,7 @@
     </row>
     <row r="61">
       <c r="A61" s="3" t="n">
-        <v>550</v>
+        <v>559</v>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
@@ -18312,7 +18600,7 @@
     </row>
     <row r="62">
       <c r="A62" s="3" t="n">
-        <v>551</v>
+        <v>560</v>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
@@ -18344,7 +18632,7 @@
     </row>
     <row r="63">
       <c r="A63" s="3" t="n">
-        <v>552</v>
+        <v>561</v>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
@@ -18376,7 +18664,7 @@
     </row>
     <row r="64">
       <c r="A64" s="3" t="n">
-        <v>553</v>
+        <v>562</v>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
@@ -18408,7 +18696,7 @@
     </row>
     <row r="65">
       <c r="A65" s="3" t="n">
-        <v>554</v>
+        <v>563</v>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
@@ -18440,7 +18728,7 @@
     </row>
     <row r="66">
       <c r="A66" s="3" t="n">
-        <v>555</v>
+        <v>564</v>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
@@ -18472,7 +18760,7 @@
     </row>
     <row r="67">
       <c r="A67" s="3" t="n">
-        <v>556</v>
+        <v>565</v>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
@@ -18504,7 +18792,7 @@
     </row>
     <row r="68">
       <c r="A68" s="3" t="n">
-        <v>557</v>
+        <v>566</v>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
@@ -18536,7 +18824,7 @@
     </row>
     <row r="69">
       <c r="A69" s="3" t="n">
-        <v>558</v>
+        <v>567</v>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
@@ -18568,7 +18856,7 @@
     </row>
     <row r="70">
       <c r="A70" s="3" t="n">
-        <v>559</v>
+        <v>568</v>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
@@ -18600,7 +18888,7 @@
     </row>
     <row r="71">
       <c r="A71" s="3" t="n">
-        <v>560</v>
+        <v>569</v>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
@@ -18632,7 +18920,7 @@
     </row>
     <row r="72">
       <c r="A72" s="3" t="n">
-        <v>561</v>
+        <v>570</v>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
@@ -18664,7 +18952,7 @@
     </row>
     <row r="73">
       <c r="A73" s="3" t="n">
-        <v>562</v>
+        <v>571</v>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
@@ -18696,7 +18984,7 @@
     </row>
     <row r="74">
       <c r="A74" s="3" t="n">
-        <v>563</v>
+        <v>572</v>
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
@@ -18728,11 +19016,11 @@
     </row>
     <row r="75">
       <c r="A75" s="3" t="n">
-        <v>564</v>
+        <v>573</v>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Page not found</t>
+          <t>30-day follow-up page</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
@@ -18742,29 +19030,29 @@
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Page not found · The Monday After</t>
+          <t>Did you do it? · The Monday After</t>
         </is>
       </c>
       <c r="E75" s="4" t="inlineStr"/>
       <c r="F75" s="3" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
-          <t>site/404.html</t>
+          <t>site/followup.html</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;Page not found \u00b7 The Monday After&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;Did you do it? \u00b7 The Monday After&lt;"}</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="n">
-        <v>565</v>
+        <v>574</v>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>Page not found</t>
+          <t>30-day follow-up page</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
@@ -18781,7 +19069,7 @@
       <c r="F76" s="3" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
-          <t>site/404.html</t>
+          <t>site/followup.html</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -18792,127 +19080,607 @@
     </row>
     <row r="77">
       <c r="A77" s="3" t="n">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>Page not found</t>
+          <t>30-day follow-up page</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>paragraph</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>Monday, 09:00</t>
+          <t>30 days on</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr"/>
       <c r="F77" s="3" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
-          <t>site/404.html</t>
+          <t>site/followup.html</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;Monday, 09:00&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;30 days on&lt;"}</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="n">
-        <v>567</v>
+        <v>576</v>
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>Page not found</t>
+          <t>30-day follow-up page</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>heading</t>
+          <t>paragraph</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>This page isn't here.</t>
+          <t>Checking your link…</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr"/>
       <c r="F78" s="3" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
-          <t>site/404.html</t>
+          <t>site/followup.html</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;This page isn't here.&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;Checking your link\u2026&lt;"}</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="n">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>Page not found</t>
+          <t>30-day follow-up page</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>paragraph</t>
+          <t>heading</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>The address may be mistyped, or the page has moved. If you came from a Monday After email, try its link again.</t>
+          <t>Did you do it?</t>
         </is>
       </c>
       <c r="E79" s="4" t="inlineStr"/>
       <c r="F79" s="3" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
-          <t>site/404.html</t>
+          <t>site/followup.html</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;The address may be mistyped, or the page has moved. If you came from a Monday After email, try its link again.&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;Did you do it?&lt;"}</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="n">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>Page not found</t>
+          <t>30-day follow-up page</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>link</t>
+          <t>paragraph</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Go to The Monday After</t>
+          <t>30 days ago, you chose one thing to take back.</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr"/>
       <c r="F80" s="3" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
+          <t>site/followup.html</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>{"kind": "text", "raw": "&gt;30 days ago, you chose one thing to take back.&lt;"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="n">
+        <v>579</v>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>30-day follow-up page</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>heading</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>You said you'd take this back</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr"/>
+      <c r="F81" s="3" t="inlineStr"/>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>site/followup.html</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>{"kind": "text", "raw": "&gt;You said you'd take this back&lt;"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="n">
+        <v>580</v>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>30-day follow-up page</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>paragraph</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>Choose one. You can change it while this link works.</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="inlineStr"/>
+      <c r="F82" s="3" t="inlineStr"/>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>site/followup.html</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>{"kind": "text", "raw": "&gt;Choose one. You can change it while this link works.&lt;"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="n">
+        <v>581</v>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>30-day follow-up page</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>button</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>Yes, I did it</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="inlineStr"/>
+      <c r="F83" s="3" t="inlineStr"/>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>site/followup.html</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>{"kind": "text", "raw": "&gt;Yes, I did it&lt;"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="n">
+        <v>582</v>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>30-day follow-up page</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>button</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>Partly</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr"/>
+      <c r="F84" s="3" t="inlineStr"/>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>site/followup.html</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>{"kind": "text", "raw": "&gt;Partly&lt;"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="n">
+        <v>583</v>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>30-day follow-up page</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>button</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>Not yet</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr"/>
+      <c r="F85" s="3" t="inlineStr"/>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>site/followup.html</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>{"kind": "text", "raw": "&gt;Not yet&lt;"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="n">
+        <v>584</v>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>30-day follow-up page</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>heading</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>Thanks.</t>
+        </is>
+      </c>
+      <c r="E86" s="4" t="inlineStr"/>
+      <c r="F86" s="3" t="inlineStr"/>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>site/followup.html</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>{"kind": "text", "raw": "&gt;Thanks.&lt;"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="n">
+        <v>585</v>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>30-day follow-up page</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>paragraph</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>That's saved with your answers for this file.</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="inlineStr"/>
+      <c r="F87" s="3" t="inlineStr"/>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>site/followup.html</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>{"kind": "text", "raw": "&gt;That's saved with your answers for this file.&lt;"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="n">
+        <v>586</v>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>30-day follow-up page</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>heading</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>Use the link in your email.</t>
+        </is>
+      </c>
+      <c r="E88" s="4" t="inlineStr"/>
+      <c r="F88" s="3" t="inlineStr"/>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>site/followup.html</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>{"kind": "text", "raw": "&gt;Use the link in your email.&lt;"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="n">
+        <v>587</v>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>30-day follow-up page</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>paragraph</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>This page opens from the link in your 30-day follow-up email.</t>
+        </is>
+      </c>
+      <c r="E89" s="4" t="inlineStr"/>
+      <c r="F89" s="3" t="inlineStr"/>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>site/followup.html</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>{"kind": "text", "raw": "&gt;This page opens from the link in your 30-day follow-up email.&lt;"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="n">
+        <v>588</v>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>Page not found</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>browser tab title</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>Page not found · The Monday After</t>
+        </is>
+      </c>
+      <c r="E90" s="4" t="inlineStr"/>
+      <c r="F90" s="3" t="inlineStr"/>
+      <c r="G90" t="inlineStr">
+        <is>
           <t>site/404.html</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr">
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>{"kind": "text", "raw": "&gt;Page not found \u00b7 The Monday After&lt;"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="n">
+        <v>589</v>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>Page not found</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>The Monday After</t>
+        </is>
+      </c>
+      <c r="E91" s="4" t="inlineStr"/>
+      <c r="F91" s="3" t="inlineStr"/>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>site/404.html</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>{"kind": "text", "raw": "&gt;The Monday After&lt;"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="n">
+        <v>590</v>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>Page not found</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>paragraph</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>Monday, 09:00</t>
+        </is>
+      </c>
+      <c r="E92" s="4" t="inlineStr"/>
+      <c r="F92" s="3" t="inlineStr"/>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>site/404.html</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>{"kind": "text", "raw": "&gt;Monday, 09:00&lt;"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="n">
+        <v>591</v>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>Page not found</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>heading</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>This page isn't here.</t>
+        </is>
+      </c>
+      <c r="E93" s="4" t="inlineStr"/>
+      <c r="F93" s="3" t="inlineStr"/>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>site/404.html</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>{"kind": "text", "raw": "&gt;This page isn't here.&lt;"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="n">
+        <v>592</v>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>Page not found</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>paragraph</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>The address may be mistyped, or the page has moved. If you came from a Monday After email, try its link again.</t>
+        </is>
+      </c>
+      <c r="E94" s="4" t="inlineStr"/>
+      <c r="F94" s="3" t="inlineStr"/>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>site/404.html</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>{"kind": "text", "raw": "&gt;The address may be mistyped, or the page has moved. If you came from a Monday After email, try its link again.&lt;"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="n">
+        <v>593</v>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>Page not found</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>Go to The Monday After</t>
+        </is>
+      </c>
+      <c r="E95" s="4" t="inlineStr"/>
+      <c r="F95" s="3" t="inlineStr"/>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>site/404.html</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
         <is>
           <t>{"kind": "text", "raw": "&gt;Go to The Monday After&lt;"}</t>
         </is>
@@ -18929,7 +19697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -18986,7 +19754,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
-        <v>570</v>
+        <v>594</v>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
@@ -19018,7 +19786,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
-        <v>571</v>
+        <v>595</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
@@ -19050,7 +19818,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
-        <v>572</v>
+        <v>596</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
@@ -19082,7 +19850,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
-        <v>573</v>
+        <v>597</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -19114,7 +19882,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
-        <v>574</v>
+        <v>598</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
@@ -19146,7 +19914,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
-        <v>575</v>
+        <v>599</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
@@ -19178,7 +19946,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
-        <v>576</v>
+        <v>600</v>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
@@ -19210,7 +19978,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
-        <v>577</v>
+        <v>601</v>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
@@ -19242,7 +20010,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
-        <v>578</v>
+        <v>602</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
@@ -19274,7 +20042,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
-        <v>579</v>
+        <v>603</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
@@ -19306,7 +20074,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
-        <v>580</v>
+        <v>604</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
@@ -19338,7 +20106,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
-        <v>581</v>
+        <v>605</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
@@ -19370,7 +20138,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
-        <v>582</v>
+        <v>606</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
@@ -19402,7 +20170,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
-        <v>583</v>
+        <v>607</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
@@ -19429,6 +20197,166 @@
       <c r="H15" t="inlineStr">
         <is>
           <t>{"kind": "code", "raw": "\" team can't read your flight recorder.\""}</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>608</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>30-day follow-up email · subject (then the file name)</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Did you do it? </t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr"/>
+      <c r="F16" s="3" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>backend/src/emails.ts</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>{"kind": "code", "raw": "\"Did you do it? \""}</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>609</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>30-day follow-up email (then the file name)</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30 days ago, at the end of </t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>backend/src/emails.ts</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>{"kind": "code", "raw": "\"30 days ago, at the end of \""}</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>610</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>30-day follow-up email (then the action)</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>, you chose one thing to take back:</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr"/>
+      <c r="F18" s="3" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>backend/src/emails.ts</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>{"kind": "code", "raw": "\", you chose one thing to take back:\""}</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>611</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>30-day follow-up email (then the link)</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Did you do it? Tell us with one tap:</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>backend/src/emails.ts</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>{"kind": "code", "raw": "\"Did you do it? Tell us with one tap:\""}</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>612</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>30-day follow-up email</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Your answer is kept with your other answers for this file. This is the only reminder we'll send about it.</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr"/>
+      <c r="F20" s="3" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>backend/src/emails.ts</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>{"kind": "code", "raw": "\"Your answer is kept with your other answers for this file. This is the only reminder we'll send about it.\""}</t>
         </is>
       </c>
     </row>
@@ -19500,7 +20428,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
-        <v>584</v>
+        <v>613</v>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
@@ -19532,7 +20460,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
-        <v>585</v>
+        <v>614</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
@@ -19564,7 +20492,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
-        <v>586</v>
+        <v>615</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
@@ -19596,7 +20524,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
-        <v>587</v>
+        <v>616</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -19628,7 +20556,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
-        <v>588</v>
+        <v>617</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
@@ -19660,7 +20588,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
-        <v>589</v>
+        <v>618</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
@@ -19692,7 +20620,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
-        <v>590</v>
+        <v>619</v>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
@@ -19724,7 +20652,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
-        <v>591</v>
+        <v>620</v>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
@@ -19756,7 +20684,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
-        <v>592</v>
+        <v>621</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
@@ -19788,7 +20716,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
-        <v>593</v>
+        <v>622</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
@@ -19820,7 +20748,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
-        <v>594</v>
+        <v>623</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
@@ -19852,7 +20780,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
-        <v>595</v>
+        <v>624</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
@@ -19884,7 +20812,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
-        <v>596</v>
+        <v>625</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
@@ -19916,7 +20844,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
-        <v>597</v>
+        <v>626</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
@@ -19930,7 +20858,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>&lt;b&gt;Your email address&lt;/b&gt;, so we can send you each monthly incident file, confirm that you signed up, and send anything you ask for, such as a copy of your flight recorder.</t>
+          <t>&lt;b&gt;Your email address&lt;/b&gt;, so we can send you each monthly incident file, confirm that you signed up, and send anything you ask for, such as a copy of your flight recorder, or the one email 30 days later asking whether you did the thing you chose to take back.</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr"/>
@@ -19942,13 +20870,13 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;&lt;b&gt;Your email address&lt;/b&gt;, so we can send you each monthly incident file, confirm that you signed up, and send anything you ask for, such as a copy of your flight recorder.&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;&lt;b&gt;Your email address&lt;/b&gt;, so we can send you each monthly incident file, confirm that you signed up, and send anything you ask for, such as a copy of your flight recorder, or the one email 30 days later asking whether you did the thing you chose to take back.&lt;"}</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
-        <v>598</v>
+        <v>627</v>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
@@ -19962,7 +20890,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>&lt;b&gt;Your answers in each file&lt;/b&gt;: the choices you make, the threads you open, what you flag, your forecast, and the one thing you choose to take back (with the date you picked). We keep them so you can return and change them, so we can send you reports about your own answers in future, and so we can understand how readers respond to crises and improve each scenario.</t>
+          <t>&lt;b&gt;Your answers in each file&lt;/b&gt;: the choices you make, the threads you open, what you flag, your forecast, and the one thing you choose to take back (with the date you picked and, if you asked us to check in after 30 days, whether you did it). We keep them so you can return and change them, so we can send you reports about your own answers in future, and so we can understand how readers respond to crises and improve each scenario.</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr"/>
@@ -19974,13 +20902,13 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>{"kind": "text", "raw": "&gt;&lt;b&gt;Your answers in each file&lt;/b&gt;: the choices you make, the threads you open, what you flag, your forecast, and the one thing you choose to take back (with the date you picked). We keep them so you can return and change them, so we can send you reports about your own answers in future, and so we can understand how readers respond to crises and improve each scenario.&lt;"}</t>
+          <t>{"kind": "text", "raw": "&gt;&lt;b&gt;Your answers in each file&lt;/b&gt;: the choices you make, the threads you open, what you flag, your forecast, and the one thing you choose to take back (with the date you picked and, if you asked us to check in after 30 days, whether you did it). We keep them so you can return and change them, so we can send you reports about your own answers in future, and so we can understand how readers respond to crises and improve each scenario.&lt;"}</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
-        <v>599</v>
+        <v>628</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
@@ -20012,7 +20940,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
-        <v>600</v>
+        <v>629</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
@@ -20044,7 +20972,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
-        <v>601</v>
+        <v>630</v>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
@@ -20076,7 +21004,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
-        <v>602</v>
+        <v>631</v>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
@@ -20108,7 +21036,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
-        <v>603</v>
+        <v>632</v>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
@@ -20140,7 +21068,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
-        <v>604</v>
+        <v>633</v>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
@@ -20172,7 +21100,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
-        <v>605</v>
+        <v>634</v>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
@@ -20204,7 +21132,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
-        <v>606</v>
+        <v>635</v>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
@@ -20236,7 +21164,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
-        <v>607</v>
+        <v>636</v>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
@@ -20268,7 +21196,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
-        <v>608</v>
+        <v>637</v>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
@@ -20300,7 +21228,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
-        <v>609</v>
+        <v>638</v>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
@@ -20332,7 +21260,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
-        <v>610</v>
+        <v>639</v>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
@@ -20364,7 +21292,7 @@
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
-        <v>611</v>
+        <v>640</v>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
@@ -20396,7 +21324,7 @@
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
-        <v>612</v>
+        <v>641</v>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
@@ -20428,7 +21356,7 @@
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
-        <v>613</v>
+        <v>642</v>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
@@ -20460,7 +21388,7 @@
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
-        <v>614</v>
+        <v>643</v>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
@@ -20492,7 +21420,7 @@
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
-        <v>615</v>
+        <v>644</v>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
@@ -20524,7 +21452,7 @@
     </row>
     <row r="34">
       <c r="A34" s="3" t="n">
-        <v>616</v>
+        <v>645</v>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
@@ -20556,7 +21484,7 @@
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
-        <v>617</v>
+        <v>646</v>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
@@ -20588,7 +21516,7 @@
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
-        <v>618</v>
+        <v>647</v>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
@@ -20620,7 +21548,7 @@
     </row>
     <row r="37">
       <c r="A37" s="3" t="n">
-        <v>619</v>
+        <v>648</v>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
@@ -20652,7 +21580,7 @@
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
-        <v>620</v>
+        <v>649</v>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
@@ -20684,7 +21612,7 @@
     </row>
     <row r="39">
       <c r="A39" s="3" t="n">
-        <v>621</v>
+        <v>650</v>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
@@ -20716,7 +21644,7 @@
     </row>
     <row r="40">
       <c r="A40" s="3" t="n">
-        <v>622</v>
+        <v>651</v>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
@@ -20748,7 +21676,7 @@
     </row>
     <row r="41">
       <c r="A41" s="3" t="n">
-        <v>623</v>
+        <v>652</v>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
@@ -20780,7 +21708,7 @@
     </row>
     <row r="42">
       <c r="A42" s="3" t="n">
-        <v>624</v>
+        <v>653</v>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Settle the copy choices, add one-click unsubscribe, and move the buttons to a stable main branch
- Decision rights: 'Front it' now counts as a Deposit; the deposit summary fits
  every route. Trust deposit's Monday line is route-neutral. Visibility deposit
  shows only for 'Build the list'.
- One-click unsubscribe: monthly and follow-up emails carry List-Unsubscribe
  headers pointing at an unsubscribe-only, POST-only link, kept out of logs.
- Buttons check they're run from main; the role record now allows main.
  Owner's steps in docs/main-branch.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013sc1NQj5NJsvj6XwZ9CiCJ
</commit_message>
<xml_diff>
--- a/docs/app-text.xlsx
+++ b/docs/app-text.xlsx
@@ -8114,7 +8114,7 @@
       </c>
       <c r="D237" s="3" t="inlineStr">
         <is>
-          <t>Finance and HR paid people together for the first time, and each saw the other work under pressure.</t>
+          <t>Finance, HR and IT worked the problem together, and each saw the others work under pressure.</t>
         </is>
       </c>
       <c r="E237" s="4" t="inlineStr"/>
@@ -8818,7 +8818,7 @@
       </c>
       <c r="D259" s="3" t="inlineStr">
         <is>
-          <t>You and HR settled who decides before the CEO had to ask.</t>
+          <t>The CEO asked who was leading and got one answer.</t>
         </is>
       </c>
       <c r="E259" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
Send the current file straight after confirming; Send skips readers who already have it
- confirm() sends CURRENT_FILE once, after the bounce and complaint check.
  If the check or the email fails, the reader is still confirmed and gets
  it at the next Send. The confirm page says the file is on its way.
- sendFile() skips readers with a 'sent' event for that file, so pressing
  Send again never duplicates; the summary shows how many were skipped.
- The API may read the sending health (ses:GetAccount, GetMetricData).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013sc1NQj5NJsvj6XwZ9CiCJ
</commit_message>
<xml_diff>
--- a/docs/app-text.xlsx
+++ b/docs/app-text.xlsx
@@ -14669,7 +14669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H60"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -16074,7 +16074,7 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Follow-up page · after answering Yes</t>
+          <t>Confirm page · after confirming, when the file is sent (after the file name)</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
@@ -16084,7 +16084,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>You did it.</t>
+          <t xml:space="preserve"> is on its way to your inbox. If it hasn't arrived in a few minutes, check your spam folder.</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr"/>
@@ -16096,7 +16096,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\"You did it.\""}</t>
+          <t>{"kind": "code", "raw": "\" is on its way to your inbox. If it hasn't arrived in a few minutes, check your spam folder.\""}</t>
         </is>
       </c>
     </row>
@@ -16106,7 +16106,7 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Follow-up page · after answering Partly</t>
+          <t>Follow-up page · after answering Yes</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
@@ -16116,7 +16116,7 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>You did part of it.</t>
+          <t>You did it.</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr"/>
@@ -16128,7 +16128,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\"You did part of it.\""}</t>
+          <t>{"kind": "code", "raw": "\"You did it.\""}</t>
         </is>
       </c>
     </row>
@@ -16138,7 +16138,7 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Follow-up page · after answering Not yet</t>
+          <t>Follow-up page · after answering Partly</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -16148,7 +16148,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Not yet.</t>
+          <t>You did part of it.</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr"/>
@@ -16160,7 +16160,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\"Not yet.\""}</t>
+          <t>{"kind": "code", "raw": "\"You did part of it.\""}</t>
         </is>
       </c>
     </row>
@@ -16170,7 +16170,7 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Follow-up page · after answering (end)</t>
+          <t>Follow-up page · after answering Not yet</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -16180,7 +16180,7 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> That's saved with your answers for this file.</t>
+          <t>Not yet.</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr"/>
@@ -16192,7 +16192,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\" That's saved with your answers for this file.\""}</t>
+          <t>{"kind": "code", "raw": "\"Not yet.\""}</t>
         </is>
       </c>
     </row>
@@ -16202,7 +16202,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Follow-up page (then the file name)</t>
+          <t>Follow-up page · after answering (end)</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -16212,7 +16212,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">30 days ago, at the end of </t>
+          <t xml:space="preserve"> That's saved with your answers for this file.</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr"/>
@@ -16224,7 +16224,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\"30 days ago, at the end of \""}</t>
+          <t>{"kind": "code", "raw": "\" That's saved with your answers for this file.\""}</t>
         </is>
       </c>
     </row>
@@ -16234,7 +16234,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Follow-up page (end)</t>
+          <t>Follow-up page (then the file name)</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -16244,7 +16244,7 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>, you chose one thing to take back.</t>
+          <t xml:space="preserve">30 days ago, at the end of </t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr"/>
@@ -16256,7 +16256,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\", you chose one thing to take back.\""}</t>
+          <t>{"kind": "code", "raw": "\"30 days ago, at the end of \""}</t>
         </is>
       </c>
     </row>
@@ -16266,7 +16266,7 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Follow-up page · answers deleted</t>
+          <t>Follow-up page (end)</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -16276,19 +16276,19 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>There's nothing to answer for this file any more.</t>
+          <t>, you chose one thing to take back.</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr"/>
       <c r="F50" s="3" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>backend/src/service.ts</t>
+          <t>site/js/pages.js</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\"There's nothing to answer for this file any more.\""}</t>
+          <t>{"kind": "code", "raw": "\", you chose one thing to take back.\""}</t>
         </is>
       </c>
     </row>
@@ -16298,7 +16298,7 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Follow-up page</t>
+          <t>Follow-up page · answers deleted</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -16308,7 +16308,7 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Please choose one of the answers.</t>
+          <t>There's nothing to answer for this file any more.</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr"/>
@@ -16320,7 +16320,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\"Please choose one of the answers.\""}</t>
+          <t>{"kind": "code", "raw": "\"There's nothing to answer for this file any more.\""}</t>
         </is>
       </c>
     </row>
@@ -16330,7 +16330,7 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Message · expired link</t>
+          <t>Follow-up page</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
@@ -16340,7 +16340,7 @@
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>This link has expired or isn't valid. Reply to any Monday After email and we'll send you a fresh one.</t>
+          <t>Please choose one of the answers.</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr"/>
@@ -16352,7 +16352,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\"This link has expired or isn't valid. Reply to any Monday After email and we'll send you a fresh one.\""}</t>
+          <t>{"kind": "code", "raw": "\"Please choose one of the answers.\""}</t>
         </is>
       </c>
     </row>
@@ -16362,7 +16362,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Message · too many tries</t>
+          <t>Message · expired link</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
@@ -16372,7 +16372,7 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Too many requests. Please wait a little and try again.</t>
+          <t>This link has expired or isn't valid. Reply to any Monday After email and we'll send you a fresh one.</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr"/>
@@ -16384,7 +16384,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\"Too many requests. Please wait a little and try again.\""}</t>
+          <t>{"kind": "code", "raw": "\"This link has expired or isn't valid. Reply to any Monday After email and we'll send you a fresh one.\""}</t>
         </is>
       </c>
     </row>
@@ -16394,7 +16394,7 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Sign-up page · busy</t>
+          <t>Message · too many tries</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
@@ -16404,7 +16404,7 @@
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>We're getting a lot of sign-ups right now. Please try again in an hour.</t>
+          <t>Too many requests. Please wait a little and try again.</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr"/>
@@ -16416,7 +16416,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\"We're getting a lot of sign-ups right now. Please try again in an hour.\""}</t>
+          <t>{"kind": "code", "raw": "\"Too many requests. Please wait a little and try again.\""}</t>
         </is>
       </c>
     </row>
@@ -16426,7 +16426,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>App · email me my flight recorder, nothing saved</t>
+          <t>Sign-up page · busy</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
@@ -16436,7 +16436,7 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>There's no saved flight recorder for this file.</t>
+          <t>We're getting a lot of sign-ups right now. Please try again in an hour.</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr"/>
@@ -16448,7 +16448,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\"There's no saved flight recorder for this file.\""}</t>
+          <t>{"kind": "code", "raw": "\"We're getting a lot of sign-ups right now. Please try again in an hour.\""}</t>
         </is>
       </c>
     </row>
@@ -16458,7 +16458,7 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Manage page</t>
+          <t>App · email me my flight recorder, nothing saved</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
@@ -16468,7 +16468,7 @@
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>You're unsubscribed, so there's nothing to pause.</t>
+          <t>There's no saved flight recorder for this file.</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr"/>
@@ -16480,7 +16480,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\"You're unsubscribed, so there's nothing to pause.\""}</t>
+          <t>{"kind": "code", "raw": "\"There's no saved flight recorder for this file.\""}</t>
         </is>
       </c>
     </row>
@@ -16490,7 +16490,7 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Sign-up page · empty email</t>
+          <t>Manage page</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
@@ -16500,19 +16500,19 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Email is missing</t>
+          <t>You're unsubscribed, so there's nothing to pause.</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr"/>
       <c r="F57" s="3" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>backend/src/validate.ts</t>
+          <t>backend/src/service.ts</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\"Email is missing\""}</t>
+          <t>{"kind": "code", "raw": "\"You're unsubscribed, so there's nothing to pause.\""}</t>
         </is>
       </c>
     </row>
@@ -16522,7 +16522,7 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Sign-up page · bad email</t>
+          <t>Sign-up page · empty email</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
@@ -16532,7 +16532,7 @@
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>That doesn't look like an email address</t>
+          <t>Email is missing</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr"/>
@@ -16544,7 +16544,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\"That doesn't look like an email address\""}</t>
+          <t>{"kind": "code", "raw": "\"Email is missing\""}</t>
         </is>
       </c>
     </row>
@@ -16554,7 +16554,7 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Flight recorder · too long (then a number)</t>
+          <t>Sign-up page · bad email</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -16564,7 +16564,7 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Please keep each entry under </t>
+          <t>That doesn't look like an email address</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr"/>
@@ -16576,7 +16576,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>{"kind": "code", "raw": "\"Please keep each entry under \""}</t>
+          <t>{"kind": "code", "raw": "\"That doesn't look like an email address\""}</t>
         </is>
       </c>
     </row>
@@ -16586,7 +16586,7 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Flight recorder · first hour empty</t>
+          <t>Flight recorder · too long (then a number)</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
@@ -16596,7 +16596,7 @@
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Please write something for the first hour</t>
+          <t xml:space="preserve">Please keep each entry under </t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr"/>
@@ -16607,6 +16607,38 @@
         </is>
       </c>
       <c r="H60" t="inlineStr">
+        <is>
+          <t>{"kind": "code", "raw": "\"Please keep each entry under \""}</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Flight recorder · first hour empty</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>Please write something for the first hour</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr"/>
+      <c r="F61" s="3" t="inlineStr"/>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>backend/src/validate.ts</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
         <is>
           <t>{"kind": "code", "raw": "\"Please write something for the first hour\""}</t>
         </is>
@@ -16680,7 +16712,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
@@ -16712,7 +16744,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
@@ -16744,7 +16776,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
@@ -16776,7 +16808,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -16808,7 +16840,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
@@ -16840,7 +16872,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
@@ -16872,7 +16904,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
@@ -16904,7 +16936,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
@@ -16936,7 +16968,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
@@ -16968,7 +17000,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
@@ -17000,7 +17032,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
@@ -17032,7 +17064,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
@@ -17064,7 +17096,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
@@ -17096,7 +17128,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
@@ -17128,7 +17160,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
@@ -17160,7 +17192,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
@@ -17192,7 +17224,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
@@ -17224,7 +17256,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
@@ -17256,7 +17288,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
@@ -17288,7 +17320,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
@@ -17320,7 +17352,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
@@ -17352,7 +17384,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
@@ -17384,7 +17416,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
@@ -17416,7 +17448,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
@@ -17448,7 +17480,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
@@ -17480,7 +17512,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
@@ -17512,7 +17544,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
@@ -17544,7 +17576,7 @@
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
@@ -17576,7 +17608,7 @@
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
@@ -17608,7 +17640,7 @@
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
@@ -17640,7 +17672,7 @@
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
@@ -17672,7 +17704,7 @@
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
@@ -17704,7 +17736,7 @@
     </row>
     <row r="34">
       <c r="A34" s="3" t="n">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
@@ -17736,7 +17768,7 @@
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
@@ -17768,7 +17800,7 @@
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
@@ -17800,7 +17832,7 @@
     </row>
     <row r="37">
       <c r="A37" s="3" t="n">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
@@ -17832,7 +17864,7 @@
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
@@ -17864,7 +17896,7 @@
     </row>
     <row r="39">
       <c r="A39" s="3" t="n">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
@@ -17896,7 +17928,7 @@
     </row>
     <row r="40">
       <c r="A40" s="3" t="n">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
@@ -17928,7 +17960,7 @@
     </row>
     <row r="41">
       <c r="A41" s="3" t="n">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
@@ -17960,7 +17992,7 @@
     </row>
     <row r="42">
       <c r="A42" s="3" t="n">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
@@ -17992,7 +18024,7 @@
     </row>
     <row r="43">
       <c r="A43" s="3" t="n">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
@@ -18024,7 +18056,7 @@
     </row>
     <row r="44">
       <c r="A44" s="3" t="n">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
@@ -18056,7 +18088,7 @@
     </row>
     <row r="45">
       <c r="A45" s="3" t="n">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
@@ -18088,7 +18120,7 @@
     </row>
     <row r="46">
       <c r="A46" s="3" t="n">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
@@ -18120,7 +18152,7 @@
     </row>
     <row r="47">
       <c r="A47" s="3" t="n">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
@@ -18152,7 +18184,7 @@
     </row>
     <row r="48">
       <c r="A48" s="3" t="n">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
@@ -18184,7 +18216,7 @@
     </row>
     <row r="49">
       <c r="A49" s="3" t="n">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
@@ -18216,7 +18248,7 @@
     </row>
     <row r="50">
       <c r="A50" s="3" t="n">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
@@ -18248,7 +18280,7 @@
     </row>
     <row r="51">
       <c r="A51" s="3" t="n">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
@@ -18280,7 +18312,7 @@
     </row>
     <row r="52">
       <c r="A52" s="3" t="n">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
@@ -18312,7 +18344,7 @@
     </row>
     <row r="53">
       <c r="A53" s="3" t="n">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
@@ -18344,7 +18376,7 @@
     </row>
     <row r="54">
       <c r="A54" s="3" t="n">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
@@ -18376,7 +18408,7 @@
     </row>
     <row r="55">
       <c r="A55" s="3" t="n">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
@@ -18408,7 +18440,7 @@
     </row>
     <row r="56">
       <c r="A56" s="3" t="n">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
@@ -18440,7 +18472,7 @@
     </row>
     <row r="57">
       <c r="A57" s="3" t="n">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
@@ -18472,7 +18504,7 @@
     </row>
     <row r="58">
       <c r="A58" s="3" t="n">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
@@ -18504,7 +18536,7 @@
     </row>
     <row r="59">
       <c r="A59" s="3" t="n">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
@@ -18536,7 +18568,7 @@
     </row>
     <row r="60">
       <c r="A60" s="3" t="n">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
@@ -18568,7 +18600,7 @@
     </row>
     <row r="61">
       <c r="A61" s="3" t="n">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
@@ -18600,7 +18632,7 @@
     </row>
     <row r="62">
       <c r="A62" s="3" t="n">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
@@ -18632,7 +18664,7 @@
     </row>
     <row r="63">
       <c r="A63" s="3" t="n">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
@@ -18664,7 +18696,7 @@
     </row>
     <row r="64">
       <c r="A64" s="3" t="n">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
@@ -18696,7 +18728,7 @@
     </row>
     <row r="65">
       <c r="A65" s="3" t="n">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
@@ -18728,7 +18760,7 @@
     </row>
     <row r="66">
       <c r="A66" s="3" t="n">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
@@ -18760,7 +18792,7 @@
     </row>
     <row r="67">
       <c r="A67" s="3" t="n">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
@@ -18792,7 +18824,7 @@
     </row>
     <row r="68">
       <c r="A68" s="3" t="n">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
@@ -18824,7 +18856,7 @@
     </row>
     <row r="69">
       <c r="A69" s="3" t="n">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
@@ -18856,7 +18888,7 @@
     </row>
     <row r="70">
       <c r="A70" s="3" t="n">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
@@ -18888,7 +18920,7 @@
     </row>
     <row r="71">
       <c r="A71" s="3" t="n">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
@@ -18920,7 +18952,7 @@
     </row>
     <row r="72">
       <c r="A72" s="3" t="n">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
@@ -18952,7 +18984,7 @@
     </row>
     <row r="73">
       <c r="A73" s="3" t="n">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
@@ -18984,7 +19016,7 @@
     </row>
     <row r="74">
       <c r="A74" s="3" t="n">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
@@ -19016,7 +19048,7 @@
     </row>
     <row r="75">
       <c r="A75" s="3" t="n">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
@@ -19048,7 +19080,7 @@
     </row>
     <row r="76">
       <c r="A76" s="3" t="n">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
@@ -19080,7 +19112,7 @@
     </row>
     <row r="77">
       <c r="A77" s="3" t="n">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
@@ -19112,7 +19144,7 @@
     </row>
     <row r="78">
       <c r="A78" s="3" t="n">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
@@ -19144,7 +19176,7 @@
     </row>
     <row r="79">
       <c r="A79" s="3" t="n">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
@@ -19176,7 +19208,7 @@
     </row>
     <row r="80">
       <c r="A80" s="3" t="n">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
@@ -19208,7 +19240,7 @@
     </row>
     <row r="81">
       <c r="A81" s="3" t="n">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
@@ -19240,7 +19272,7 @@
     </row>
     <row r="82">
       <c r="A82" s="3" t="n">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
@@ -19272,7 +19304,7 @@
     </row>
     <row r="83">
       <c r="A83" s="3" t="n">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
@@ -19304,7 +19336,7 @@
     </row>
     <row r="84">
       <c r="A84" s="3" t="n">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
@@ -19336,7 +19368,7 @@
     </row>
     <row r="85">
       <c r="A85" s="3" t="n">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
@@ -19368,7 +19400,7 @@
     </row>
     <row r="86">
       <c r="A86" s="3" t="n">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
@@ -19400,7 +19432,7 @@
     </row>
     <row r="87">
       <c r="A87" s="3" t="n">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
@@ -19432,7 +19464,7 @@
     </row>
     <row r="88">
       <c r="A88" s="3" t="n">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
@@ -19464,7 +19496,7 @@
     </row>
     <row r="89">
       <c r="A89" s="3" t="n">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
@@ -19496,7 +19528,7 @@
     </row>
     <row r="90">
       <c r="A90" s="3" t="n">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
@@ -19528,7 +19560,7 @@
     </row>
     <row r="91">
       <c r="A91" s="3" t="n">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
@@ -19560,7 +19592,7 @@
     </row>
     <row r="92">
       <c r="A92" s="3" t="n">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
@@ -19592,7 +19624,7 @@
     </row>
     <row r="93">
       <c r="A93" s="3" t="n">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
@@ -19624,7 +19656,7 @@
     </row>
     <row r="94">
       <c r="A94" s="3" t="n">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
@@ -19656,7 +19688,7 @@
     </row>
     <row r="95">
       <c r="A95" s="3" t="n">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
@@ -19754,7 +19786,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
@@ -19786,7 +19818,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
@@ -19818,7 +19850,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
@@ -19850,7 +19882,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -19882,7 +19914,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
@@ -19914,7 +19946,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
@@ -19946,7 +19978,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
@@ -19978,7 +20010,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
@@ -20010,7 +20042,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
@@ -20042,7 +20074,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
@@ -20074,7 +20106,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
@@ -20106,7 +20138,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
@@ -20138,7 +20170,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
@@ -20170,7 +20202,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
@@ -20202,7 +20234,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
@@ -20234,7 +20266,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
@@ -20266,7 +20298,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
@@ -20298,7 +20330,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
@@ -20330,7 +20362,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
@@ -20428,7 +20460,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
@@ -20460,7 +20492,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
@@ -20492,7 +20524,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
@@ -20524,7 +20556,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -20556,7 +20588,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
@@ -20588,7 +20620,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
@@ -20620,7 +20652,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
@@ -20652,7 +20684,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
@@ -20684,7 +20716,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
@@ -20716,7 +20748,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
@@ -20748,7 +20780,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
@@ -20780,7 +20812,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
@@ -20812,7 +20844,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
@@ -20844,7 +20876,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
@@ -20876,7 +20908,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
@@ -20908,7 +20940,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
@@ -20940,7 +20972,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
@@ -20972,7 +21004,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
@@ -21004,7 +21036,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
@@ -21036,7 +21068,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
@@ -21068,7 +21100,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
@@ -21100,7 +21132,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
@@ -21132,7 +21164,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
@@ -21164,7 +21196,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
@@ -21196,7 +21228,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
@@ -21228,7 +21260,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
@@ -21260,7 +21292,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
@@ -21292,7 +21324,7 @@
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
@@ -21324,7 +21356,7 @@
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
@@ -21356,7 +21388,7 @@
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
@@ -21388,7 +21420,7 @@
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
@@ -21420,7 +21452,7 @@
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
@@ -21452,7 +21484,7 @@
     </row>
     <row r="34">
       <c r="A34" s="3" t="n">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
@@ -21484,7 +21516,7 @@
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
@@ -21516,7 +21548,7 @@
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
@@ -21548,7 +21580,7 @@
     </row>
     <row r="37">
       <c r="A37" s="3" t="n">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
@@ -21580,7 +21612,7 @@
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
@@ -21612,7 +21644,7 @@
     </row>
     <row r="39">
       <c r="A39" s="3" t="n">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
@@ -21644,7 +21676,7 @@
     </row>
     <row r="40">
       <c r="A40" s="3" t="n">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
@@ -21676,7 +21708,7 @@
     </row>
     <row r="41">
       <c r="A41" s="3" t="n">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
@@ -21708,7 +21740,7 @@
     </row>
     <row r="42">
       <c r="A42" s="3" t="n">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>

</xml_diff>